<commit_message>
prep: data fixes from audit (pre-challenge)
- W007: add 'وحفص تركوه، ومنهم من كذبه'; note: the witness does not strengthen the hadith
- W019: attribute weakening to 'شيخنا' (Ibn Hajar) as transmitted by Sakhawi (p.259); add Ibn al-Jawzi (Mawdu'at) and Daraqutni 'لا يثبت منها شيء'
- Q001/Q002 regenerated from data/quran/quran-uthmani.txt without U+06DD (Q006 aligned)
- review sheet regenerated; dropdown still نعم/لا/تعديل (apply_review.py unchanged)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/review/review_sheet.xlsx
+++ b/review/review_sheet.xlsx
@@ -1191,8 +1191,8 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>ذكر السخاوي للحديث شاهداً من حديث ابن عمر بلفظ آخر، ورجاله «من أهل الصدق» لكن فيه تدليس بقية؛ ولا يُنقل حكمه على اللفظ المشهور
-رواية متصلة: من بدأكم بالكلام قبل السلام فلا تجيبوه — وله شاهد عند أبي نُعيم في الحلية، وابن السني في عمل اليوم والليلة، من حديث بقية عن عبد العزيز بن أبي رواد عن نافع عن ابن عمر مرفوعاً: من بدأكم بالكلام قبل السلام فلا تجيبوه، ورجاله من أهل الصدق، لكن بقية مدلس وقد عنعنه</t>
+          <t>الشاهد المذكور (رواية ابن عمر بلفظ آخر) لا يقوّي الحديث: رجاله «من أهل الصدق» لكن فيه تدليس بقية، ومتابعته جاءت عن راوٍ قال السخاوي فيه «وحفص تركوه، ومنهم من كذبه». فلا يُفهم أنه يرفع الحكم عن اللفظ المشهور، ولا يُنقل حكمه عليه.
+رواية متصلة: من بدأكم بالكلام قبل السلام فلا تجيبوه — وله شاهد عند أبي نُعيم في الحلية، وابن السني في عمل اليوم والليلة، من حديث بقية عن عبد العزيز بن أبي رواد عن نافع عن ابن عمر مرفوعاً: من بدأكم بالكلام قبل السلام فلا تجيبوه، ورجاله من أهل الصدق، لكن بقية مدلس وقد عنعنه، لكن قد تابعه حفص بن عمر الأيلي عن عبد العزيز، أخرجه ابن عدي في ترجمة عبد العزيز من الكامل، وحفص تركوه، ومنهم من كذبه</t>
         </is>
       </c>
       <c r="I7" s="9" t="n"/>
@@ -1711,8 +1711,8 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>الحكم «لا أصل له» يخص صيغة «الكريم حبيب الله ولو كان فاسقاً» تحديداً. أما حديث «السخي قريب من الله…» فصيغة أخرى حكم عليها السخاوي بالضعف (ونقل عن ابن الجوزي إيراده في الموضوعات وعن شيخه أن ذلك الحكم ليس بجيد)، فلا يُسحب الحكم عليها.
-رواية متصلة: السخي قريب من اللَّه، قريب من الناس، قريب من الجنة، بعيد من النار — قال شيخنا: ولا يلزم من هذه العبارة أن يكون موضوعاً، فالثابت يشمل الصحيح، والضعيف دونه، وهذا ضعيف</t>
+          <t>الحكم «لا أصل له» يخص صيغة «الكريم حبيب الله ولو كان فاسقاً» تحديداً. أما حديث «السخي قريب من الله…» فصيغة أخرى: أورده ابن الجوزي في الموضوعات ونقل عن الدارقطني «ولا يثبت منها شيء»، وقال «شيخنا» (ابن حجر) كما نقله السخاوي إنه ضعيف وإن الحكم عليه بالوضع «ليس بجيد». فلا يُسحب الحكم على إحدى الصيغتين إلى الأخرى.
+رواية متصلة: السخي قريب من اللَّه، قريب من الناس، قريب من الجنة، بعيد من النار — ونقل ابن الجوزي في الموضوعات، لما ذكر هذا الحديث فيها عن الدارقطني أنه قال: لهذا الحديث طرق، ولا يثبت منها شيء، قال شيخنا: ولا يلزم من هذه العبارة أن يكون موضوعاً، فالثابت يشمل الصحيح، والضعيف دونه، وهذا ضعيف، فالحكم ليس بجيد عليه كما بسطه في موضع آخر</t>
         </is>
       </c>
       <c r="I19" s="9" t="n"/>
@@ -2513,12 +2513,12 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>فَإِنَّ مَعَ الْعُسْرِ يُسْرًا ۝ إِنَّ مَعَ الْعُسْرِ يُسْرًا</t>
+          <t>فَإِنَّ مَعَ ٱلْعُسْرِ يُسْرًا إِنَّ مَعَ ٱلْعُسْرِ يُسْرًا</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>القرآن الكريم (رواية حفص) — الشرح 94:5-6</t>
+          <t>القرآن الكريم (رواية حفص) — 94:5-6</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -2553,12 +2553,12 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>وَمَنْ يَتَّقِ اللَّهَ يَجْعَلْ لَهُ مَخْرَجًا ۝ وَيَرْزُقْهُ مِنْ حَيْثُ لَا يَحْتَسِبُ</t>
+          <t>وَمَن يَتَّقِ ٱللَّهَ يَجْعَل لَّهُۥ مَخْرَجًا وَيَرْزُقْهُ مِنْ حَيْثُ لَا يَحْتَسِبُ</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>القرآن الكريم (رواية حفص) — الطلاق 65:2-3</t>
+          <t>القرآن الكريم (رواية حفص) — 65:2-3 (جزء من الآيتين)</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>وَٱلْعَصْرِ ۝ إِنَّ ٱلْإِنسَٰنَ لَفِى خُسْرٍ ۝ إِلَّا ٱلَّذِينَ ءَامَنُوا۟ وَعَمِلُوا۟ ٱلصَّٰلِحَٰتِ وَتَوَاصَوْا۟ بِٱلْحَقِّ وَتَوَاصَوْا۟ بِٱلصَّبْرِ</t>
+          <t>وَٱلْعَصْرِ إِنَّ ٱلْإِنسَٰنَ لَفِى خُسْرٍ إِلَّا ٱلَّذِينَ ءَامَنُوا۟ وَعَمِلُوا۟ ٱلصَّٰلِحَٰتِ وَتَوَاصَوْا۟ بِٱلْحَقِّ وَتَوَاصَوْا۟ بِٱلصَّبْرِ</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">

</xml_diff>